<commit_message>
[UPD] Updated corrected database
</commit_message>
<xml_diff>
--- a/data/daily_manual_rain_gage_data.xlsx
+++ b/data/daily_manual_rain_gage_data.xlsx
@@ -1142,7 +1142,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E4404"/>
+  <dimension ref="A1:E4451"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -50765,7 +50765,6 @@
       <c r="C4402">
         <v>4.6</v>
       </c>
-      <c r="D4402"/>
       <c r="E4402">
         <v>1</v>
       </c>
@@ -50784,12 +50783,571 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4404" spans="1:2">
+    <row r="4404" spans="1:4">
       <c r="A4404" s="7">
         <v>4402</v>
       </c>
       <c r="B4404" s="10">
         <v>46042</v>
+      </c>
+      <c r="C4404">
+        <v>10.6</v>
+      </c>
+      <c r="D4404">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4405" spans="1:4">
+      <c r="A4405" s="7">
+        <v>4403</v>
+      </c>
+      <c r="B4405" s="10">
+        <v>46043</v>
+      </c>
+      <c r="C4405">
+        <v>3.6</v>
+      </c>
+      <c r="D4405">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4406" spans="1:4">
+      <c r="A4406" s="7">
+        <v>4404</v>
+      </c>
+      <c r="B4406" s="10">
+        <v>46044</v>
+      </c>
+      <c r="C4406">
+        <v>8.4</v>
+      </c>
+      <c r="D4406">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4407" spans="1:4">
+      <c r="A4407" s="7">
+        <v>4405</v>
+      </c>
+      <c r="B4407" s="10">
+        <v>46045</v>
+      </c>
+      <c r="C4407">
+        <v>0.2</v>
+      </c>
+      <c r="D4407">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4408" spans="1:4">
+      <c r="A4408" s="7">
+        <v>4406</v>
+      </c>
+      <c r="B4408" s="10">
+        <v>46046</v>
+      </c>
+      <c r="C4408">
+        <v>3.8</v>
+      </c>
+      <c r="D4408">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4409" spans="1:4">
+      <c r="A4409" s="7">
+        <v>4407</v>
+      </c>
+      <c r="B4409" s="10">
+        <v>46047</v>
+      </c>
+      <c r="C4409">
+        <v>0.2</v>
+      </c>
+      <c r="D4409">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4410" spans="1:3">
+      <c r="A4410" s="7">
+        <v>4408</v>
+      </c>
+      <c r="B4410" s="10">
+        <v>46048</v>
+      </c>
+      <c r="C4410">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4411" spans="1:3">
+      <c r="A4411" s="7">
+        <v>4409</v>
+      </c>
+      <c r="B4411" s="10">
+        <v>46049</v>
+      </c>
+      <c r="C4411">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="4412" spans="1:3">
+      <c r="A4412" s="7">
+        <v>4410</v>
+      </c>
+      <c r="B4412" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C4412">
+        <v>24.6</v>
+      </c>
+    </row>
+    <row r="4413" spans="1:4">
+      <c r="A4413" s="7">
+        <v>4411</v>
+      </c>
+      <c r="B4413" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C4413">
+        <v>1.2</v>
+      </c>
+      <c r="D4413">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4414" spans="1:3">
+      <c r="A4414" s="7">
+        <v>4412</v>
+      </c>
+      <c r="B4414" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C4414">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="4415" spans="1:3">
+      <c r="A4415" s="7">
+        <v>4413</v>
+      </c>
+      <c r="B4415" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C4415">
+        <v>12.6</v>
+      </c>
+    </row>
+    <row r="4416" spans="1:3">
+      <c r="A4416" s="7">
+        <v>4414</v>
+      </c>
+      <c r="B4416" s="10">
+        <v>46054</v>
+      </c>
+      <c r="C4416">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4417" spans="1:3">
+      <c r="A4417" s="7">
+        <v>4415</v>
+      </c>
+      <c r="B4417" s="10">
+        <v>46055</v>
+      </c>
+      <c r="C4417">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4418" spans="1:3">
+      <c r="A4418" s="7">
+        <v>4416</v>
+      </c>
+      <c r="B4418" s="10">
+        <v>46056</v>
+      </c>
+      <c r="C4418">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4419" spans="1:3">
+      <c r="A4419" s="7">
+        <v>4417</v>
+      </c>
+      <c r="B4419" s="10">
+        <v>46057</v>
+      </c>
+      <c r="C4419">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4420" spans="1:3">
+      <c r="A4420" s="7">
+        <v>4418</v>
+      </c>
+      <c r="B4420" s="10">
+        <v>46058</v>
+      </c>
+      <c r="C4420">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4421" spans="1:3">
+      <c r="A4421" s="7">
+        <v>4419</v>
+      </c>
+      <c r="B4421" s="10">
+        <v>46059</v>
+      </c>
+      <c r="C4421">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4422" spans="1:3">
+      <c r="A4422" s="7">
+        <v>4420</v>
+      </c>
+      <c r="B4422" s="10">
+        <v>46060</v>
+      </c>
+      <c r="C4422">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4423" spans="1:4">
+      <c r="A4423" s="7">
+        <v>4421</v>
+      </c>
+      <c r="B4423" s="10">
+        <v>46061</v>
+      </c>
+      <c r="C4423">
+        <v>2.6</v>
+      </c>
+      <c r="D4423">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4424" spans="1:3">
+      <c r="A4424" s="7">
+        <v>4422</v>
+      </c>
+      <c r="B4424" s="10">
+        <v>46062</v>
+      </c>
+      <c r="C4424">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4425" spans="1:3">
+      <c r="A4425" s="7">
+        <v>4423</v>
+      </c>
+      <c r="B4425" s="10">
+        <v>46063</v>
+      </c>
+      <c r="C4425">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4426" spans="1:3">
+      <c r="A4426" s="7">
+        <v>4424</v>
+      </c>
+      <c r="B4426" s="10">
+        <v>46064</v>
+      </c>
+      <c r="C4426">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4427" spans="1:3">
+      <c r="A4427" s="7">
+        <v>4425</v>
+      </c>
+      <c r="B4427" s="10">
+        <v>46065</v>
+      </c>
+      <c r="C4427">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4428" spans="1:4">
+      <c r="A4428" s="7">
+        <v>4426</v>
+      </c>
+      <c r="B4428" s="10">
+        <v>46066</v>
+      </c>
+      <c r="C4428">
+        <v>4</v>
+      </c>
+      <c r="D4428">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4429" spans="1:3">
+      <c r="A4429" s="7">
+        <v>4427</v>
+      </c>
+      <c r="B4429" s="10">
+        <v>46067</v>
+      </c>
+      <c r="C4429">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="4430" spans="1:3">
+      <c r="A4430" s="7">
+        <v>4428</v>
+      </c>
+      <c r="B4430" s="10">
+        <v>46068</v>
+      </c>
+      <c r="C4430">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4431" spans="1:3">
+      <c r="A4431" s="7">
+        <v>4429</v>
+      </c>
+      <c r="B4431" s="10">
+        <v>46069</v>
+      </c>
+      <c r="C4431">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4432" spans="1:3">
+      <c r="A4432" s="7">
+        <v>4430</v>
+      </c>
+      <c r="B4432" s="10">
+        <v>46070</v>
+      </c>
+      <c r="C4432">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4433" spans="1:3">
+      <c r="A4433" s="7">
+        <v>4431</v>
+      </c>
+      <c r="B4433" s="10">
+        <v>46071</v>
+      </c>
+      <c r="C4433">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4434" spans="1:3">
+      <c r="A4434" s="7">
+        <v>4432</v>
+      </c>
+      <c r="B4434" s="10">
+        <v>46072</v>
+      </c>
+      <c r="C4434">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4435" spans="1:3">
+      <c r="A4435" s="7">
+        <v>4433</v>
+      </c>
+      <c r="B4435" s="10">
+        <v>46073</v>
+      </c>
+      <c r="C4435">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4436" spans="1:3">
+      <c r="A4436" s="7">
+        <v>4434</v>
+      </c>
+      <c r="B4436" s="10">
+        <v>46074</v>
+      </c>
+      <c r="C4436">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4437" spans="1:3">
+      <c r="A4437" s="7">
+        <v>4435</v>
+      </c>
+      <c r="B4437" s="10">
+        <v>46075</v>
+      </c>
+      <c r="C4437">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4438" spans="1:3">
+      <c r="A4438" s="7">
+        <v>4436</v>
+      </c>
+      <c r="B4438" s="10">
+        <v>46076</v>
+      </c>
+      <c r="C4438">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4439" spans="1:4">
+      <c r="A4439" s="7">
+        <v>4437</v>
+      </c>
+      <c r="B4439" s="10">
+        <v>46077</v>
+      </c>
+      <c r="C4439">
+        <v>0.2</v>
+      </c>
+      <c r="D4439">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4440" spans="1:3">
+      <c r="A4440" s="7">
+        <v>4438</v>
+      </c>
+      <c r="B4440" s="10">
+        <v>46078</v>
+      </c>
+      <c r="C4440">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4441" spans="1:3">
+      <c r="A4441" s="7">
+        <v>4439</v>
+      </c>
+      <c r="B4441" s="10">
+        <v>46079</v>
+      </c>
+      <c r="C4441">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4442" spans="1:3">
+      <c r="A4442" s="7">
+        <v>4440</v>
+      </c>
+      <c r="B4442" s="10">
+        <v>46080</v>
+      </c>
+      <c r="C4442">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4443" spans="1:3">
+      <c r="A4443" s="7">
+        <v>4441</v>
+      </c>
+      <c r="B4443" s="10">
+        <v>46081</v>
+      </c>
+      <c r="C4443">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4444" spans="1:3">
+      <c r="A4444" s="7">
+        <v>4442</v>
+      </c>
+      <c r="B4444" s="10">
+        <v>46082</v>
+      </c>
+      <c r="C4444">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4445" spans="1:3">
+      <c r="A4445" s="7">
+        <v>4443</v>
+      </c>
+      <c r="B4445" s="10">
+        <v>46083</v>
+      </c>
+      <c r="C4445">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4446" spans="1:3">
+      <c r="A4446" s="7">
+        <v>4444</v>
+      </c>
+      <c r="B4446" s="10">
+        <v>46084</v>
+      </c>
+      <c r="C4446">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4447" spans="1:3">
+      <c r="A4447" s="7">
+        <v>4445</v>
+      </c>
+      <c r="B4447" s="10">
+        <v>46085</v>
+      </c>
+      <c r="C4447">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4448" spans="1:4">
+      <c r="A4448" s="7">
+        <v>4446</v>
+      </c>
+      <c r="B4448" s="10">
+        <v>46086</v>
+      </c>
+      <c r="C4448">
+        <v>9.4</v>
+      </c>
+      <c r="D4448">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4449" spans="1:4">
+      <c r="A4449" s="7">
+        <v>4447</v>
+      </c>
+      <c r="B4449" s="10">
+        <v>46087</v>
+      </c>
+      <c r="C4449">
+        <v>25</v>
+      </c>
+      <c r="D4449">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4450" spans="1:4">
+      <c r="A4450" s="7">
+        <v>4448</v>
+      </c>
+      <c r="B4450" s="10">
+        <v>46088</v>
+      </c>
+      <c r="C4450">
+        <v>12.4</v>
+      </c>
+      <c r="D4450">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4451" spans="1:3">
+      <c r="A4451" s="7">
+        <v>4449</v>
+      </c>
+      <c r="B4451" s="10">
+        <v>46089</v>
+      </c>
+      <c r="C4451">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[UPD] Updated corrected database. Changed baseline in monthly mean precipitation to 2014-2023
</commit_message>
<xml_diff>
--- a/data/daily_manual_rain_gage_data.xlsx
+++ b/data/daily_manual_rain_gage_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eiven\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eiven\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F921B943-2BBE-40A8-A51F-6BF513C8F77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{434B4394-30FD-4D99-9054-3DBCA633B0D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -145,7 +145,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -250,7 +250,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -531,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4470"/>
+  <dimension ref="A1:E4472"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -50946,6 +50946,28 @@
       </c>
       <c r="C4470">
         <v>0</v>
+      </c>
+    </row>
+    <row r="4471" spans="1:3">
+      <c r="A4471" s="7">
+        <v>4469</v>
+      </c>
+      <c r="B4471" s="10">
+        <v>46109</v>
+      </c>
+      <c r="C4471">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4472" spans="1:3">
+      <c r="A4472" s="7">
+        <v>4470</v>
+      </c>
+      <c r="B4472" s="10">
+        <v>46110</v>
+      </c>
+      <c r="C4472">
+        <v>35.200000000000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>